<commit_message>
Correct benchmark arithmetic, chronology, and legal guide
</commit_message>
<xml_diff>
--- a/participant/17_cap_table_and_dilution.xlsx
+++ b/participant/17_cap_table_and_dilution.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Rb519a24f19fe430f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Series A Closing" sheetId="2" r:id="Rbf0dfea87f5a450a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge Board Pack" sheetId="3" r:id="R46193b7ce4564dba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corrected Dilution" sheetId="4" r:id="R8dc28ae010db4e26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="R2fd96499f2994d7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R9ab5952051b64179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Series A Closing" sheetId="2" r:id="R08521a75ce5a4ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge Board Pack" sheetId="3" r:id="R2529f921f5764d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corrected Dilution" sheetId="4" r:id="Rdd948e8f0da54172"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="5" r:id="R4f360f9d2d62452a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -339,7 +339,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -350,7 +350,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -361,7 +361,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1196,7 +1196,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="D9" s="80" t="str">
-        <x:v>Board pack price differs from stated INR 1.80</x:v>
+        <x:v>Board-pack formula differs from stated INR 18.00</x:v>
       </x:c>
       <x:c r="E9" s="42"/>
       <x:c r="F9" s="42"/>
@@ -1626,7 +1626,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="41" t="str">
-        <x:v>Formula-driven reconstruction using INR 1.80 and the SHA fully diluted definition</x:v>
+        <x:v>Formula-driven reconstruction using INR 18.00 and the SHA fully diluted definition</x:v>
       </x:c>
       <x:c r="B2" s="41"/>
       <x:c r="C2" s="41"/>
@@ -1722,7 +1722,7 @@
         <x:v>Agreed price per share</x:v>
       </x:c>
       <x:c r="B9" s="87" t="n">
-        <x:v>1.8</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C9" s="42"/>
       <x:c r="D9" s="42"/>
@@ -1737,7 +1737,7 @@
       </x:c>
       <x:c r="B10" s="87" t="n">
         <x:f>B8/B9</x:f>
-        <x:v>50000000</x:v>
+        <x:v>5000000</x:v>
       </x:c>
       <x:c r="C10" s="42"/>
       <x:c r="D10" s="42"/>
@@ -2016,7 +2016,9 @@
       <x:c r="H21" s="42"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="42"/>
+      <x:c r="A22" s="42" t="str">
+        <x:v>Anti-dilution: Meridian's written 30 September waiver is specific to this bridge; no clause 7 conversion adjustment is modelled.</x:v>
+      </x:c>
       <x:c r="B22" s="42"/>
       <x:c r="C22" s="42"/>
       <x:c r="D22" s="42"/>
@@ -2393,25 +2395,66 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="42" t="str">
-        <x:v>Formula error scan</x:v>
+        <x:v>Bridge price arithmetic</x:v>
       </x:c>
       <x:c r="B12" s="79" t="n">
-        <x:v>0</x:v>
+        <x:f>'Corrected Dilution'!B8/'Corrected Dilution'!B10</x:f>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C12" s="79" t="n">
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D12" s="79" t="n">
+        <x:f>B12-C12</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="42" t="str">
+        <x:f>IF(ABS(D12)&lt;0.00001,"PASS","WARN")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F12" s="42" t="str">
-        <x:v>No spreadsheet formula errors intended</x:v>
+        <x:v>INR 90m / 5m shares</x:v>
       </x:c>
       <x:c r="G12" s="42"/>
       <x:c r="H12" s="42"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>Anti-dilution treatment</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Specific written waiver</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>No adjustment</x:v>
+      </x:c>
+      <x:c r="D13"/>
+      <x:c r="E13" t="str">
+        <x:v>INFO</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>VP-05: 30 Sep waiver; authority schedule absent</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Formula error scan</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>No spreadsheet formula errors intended</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>